<commit_message>
Agent 2 & 3 Changes and Optimizations
</commit_message>
<xml_diff>
--- a/agent-2/src/runs/stadium_leads_2026-06-23.xlsx
+++ b/agent-2/src/runs/stadium_leads_2026-06-23.xlsx
@@ -506,7 +506,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -702,16 +702,13 @@
     <xf numFmtId="0" fontId="28" fillId="33" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="34" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1596,13 +1593,13 @@
       <c r="P1" s="12" t="inlineStr">
         <is>
           <t>Tier 3
-6</t>
+8</t>
         </is>
       </c>
       <c r="Q1" s="13" t="inlineStr">
         <is>
           <t>Tier 4
-20</t>
+18</t>
         </is>
       </c>
       <c r="R1" s="14" t="inlineStr">
@@ -1684,7 +1681,7 @@
         </is>
       </c>
       <c r="Y2" s="16" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Z2" s="16" t="n"/>
       <c r="AA2" s="16" t="inlineStr">
@@ -1722,7 +1719,7 @@
         </is>
       </c>
       <c r="V3" s="16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W3" s="16" t="n"/>
       <c r="X3" s="16" t="inlineStr">
@@ -1731,7 +1728,7 @@
         </is>
       </c>
       <c r="Y3" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Z3" s="16" t="n"/>
       <c r="AA3" s="16" t="inlineStr">
@@ -1781,7 +1778,7 @@
         </is>
       </c>
       <c r="V4" s="16" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="W4" s="16" t="n"/>
       <c r="X4" s="16" t="n"/>
@@ -1802,7 +1799,7 @@
         </is>
       </c>
       <c r="AE4" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF4" s="16" t="n"/>
       <c r="AG4" s="16" t="n"/>
@@ -1873,7 +1870,7 @@
         </is>
       </c>
       <c r="AE5" s="16" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AF5" s="16" t="n"/>
       <c r="AG5" s="16" t="n"/>
@@ -1897,7 +1894,7 @@
       <c r="I6" s="24" t="n"/>
       <c r="J6" s="24" t="n"/>
       <c r="K6" s="32" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L6" s="26" t="n"/>
       <c r="M6" s="26" t="n"/>
@@ -1907,7 +1904,7 @@
       <c r="O6" s="28" t="n"/>
       <c r="P6" s="28" t="n"/>
       <c r="Q6" s="34" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R6" s="22" t="n"/>
       <c r="S6" s="22" t="n"/>
@@ -2526,16 +2523,16 @@
       </c>
       <c r="C27" s="43" t="inlineStr">
         <is>
-          <t>New Chiefs Stadium</t>
+          <t>New Dallas Arena</t>
         </is>
       </c>
       <c r="D27" s="42" t="inlineStr">
         <is>
-          <t>Kansas City, KS</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E27" s="42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="44" t="n">
         <v>60</v>
@@ -2574,7 +2571,7 @@
       </c>
       <c r="O27" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Darrell K Royal–Texas </t>
+          <t>Notre Dame Stadium</t>
         </is>
       </c>
       <c r="P27" s="48" t="inlineStr">
@@ -2601,16 +2598,16 @@
       </c>
       <c r="C28" s="53" t="inlineStr">
         <is>
-          <t>New Dallas Arena</t>
+          <t>New Chiefs Stadium</t>
         </is>
       </c>
       <c r="D28" s="52" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Kansas City, KS</t>
         </is>
       </c>
       <c r="E28" s="52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" s="44" t="n">
         <v>60</v>
@@ -2620,7 +2617,7 @@
       </c>
       <c r="H28" s="53" t="inlineStr">
         <is>
-          <t>Kyle Field</t>
+          <t>Tiger Stadium</t>
         </is>
       </c>
       <c r="I28" s="52" t="inlineStr">
@@ -2695,7 +2692,7 @@
       </c>
       <c r="H29" s="46" t="inlineStr">
         <is>
-          <t>Williams–Brice Stadium</t>
+          <t>Neyland Stadium</t>
         </is>
       </c>
       <c r="I29" s="45" t="inlineStr">
@@ -2756,7 +2753,7 @@
       </c>
       <c r="H30" s="53" t="inlineStr">
         <is>
-          <t>Neyland Stadium</t>
+          <t>Williams–Brice Stadium</t>
         </is>
       </c>
       <c r="I30" s="52" t="inlineStr">
@@ -2817,7 +2814,7 @@
       </c>
       <c r="H31" s="46" t="inlineStr">
         <is>
-          <t>Tiger Stadium</t>
+          <t>Kyle Field</t>
         </is>
       </c>
       <c r="I31" s="45" t="inlineStr">
@@ -2878,16 +2875,16 @@
       </c>
       <c r="H32" s="53" t="inlineStr">
         <is>
-          <t>Chicago Bears Stadium</t>
+          <t>Sanford Stadium</t>
         </is>
       </c>
       <c r="I32" s="52" t="inlineStr">
         <is>
-          <t>NFL</t>
+          <t>NCAA</t>
         </is>
       </c>
       <c r="J32" s="52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" s="51" t="inlineStr">
         <is>
@@ -2895,7 +2892,7 @@
         </is>
       </c>
       <c r="L32" s="52" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="M32" s="52" t="inlineStr">
         <is>
@@ -2907,7 +2904,7 @@
       </c>
       <c r="O32" s="53" t="inlineStr">
         <is>
-          <t>Future South Florida o</t>
+          <t>New Aloha Stadium</t>
         </is>
       </c>
       <c r="P32" s="52" t="inlineStr">
@@ -2939,16 +2936,16 @@
       </c>
       <c r="H33" s="46" t="inlineStr">
         <is>
-          <t>Sanford Stadium</t>
+          <t>Chicago Bears Stadium</t>
         </is>
       </c>
       <c r="I33" s="45" t="inlineStr">
         <is>
-          <t>NCAA</t>
+          <t>NFL</t>
         </is>
       </c>
       <c r="J33" s="45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K33" s="51" t="inlineStr">
         <is>
@@ -2956,7 +2953,7 @@
         </is>
       </c>
       <c r="L33" s="45" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="M33" s="45" t="inlineStr">
         <is>
@@ -2968,20 +2965,20 @@
       </c>
       <c r="O33" s="49" t="inlineStr">
         <is>
-          <t>New Broncos Stadium</t>
+          <t>Future South Florida o</t>
         </is>
       </c>
       <c r="P33" s="48" t="inlineStr">
         <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="Q33" s="58" t="n">
-        <v>4</v>
-      </c>
-      <c r="R33" s="47" t="inlineStr">
-        <is>
-          <t>Too Late</t>
+          <t>NCAA</t>
+        </is>
+      </c>
+      <c r="Q33" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="R33" s="51" t="inlineStr">
+        <is>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="S33" s="48" t="n">
@@ -3000,12 +2997,12 @@
       </c>
       <c r="H34" s="53" t="inlineStr">
         <is>
-          <t>California Memorial Stad</t>
+          <t>New South Philadelphia A</t>
         </is>
       </c>
       <c r="I34" s="52" t="inlineStr">
         <is>
-          <t>NCAA</t>
+          <t>NBA</t>
         </is>
       </c>
       <c r="J34" s="52" t="n">
@@ -3029,20 +3026,20 @@
       </c>
       <c r="O34" s="53" t="inlineStr">
         <is>
-          <t>Gaylord Family Oklahom</t>
+          <t>New Broncos Stadium</t>
         </is>
       </c>
       <c r="P34" s="52" t="inlineStr">
         <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="Q34" s="57" t="n">
-        <v>3</v>
-      </c>
-      <c r="R34" s="51" t="inlineStr">
-        <is>
-          <t>Monitor</t>
+          <t>NFL</t>
+        </is>
+      </c>
+      <c r="Q34" s="58" t="n">
+        <v>4</v>
+      </c>
+      <c r="R34" s="47" t="inlineStr">
+        <is>
+          <t>Too Late</t>
         </is>
       </c>
       <c r="S34" s="52" t="n">
@@ -3061,20 +3058,20 @@
       </c>
       <c r="H35" s="46" t="inlineStr">
         <is>
-          <t>Notre Dame Stadium</t>
+          <t>New Dallas Arena</t>
         </is>
       </c>
       <c r="I35" s="45" t="inlineStr">
         <is>
-          <t>NCAA</t>
+          <t>NBA</t>
         </is>
       </c>
       <c r="J35" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="K35" s="51" t="inlineStr">
-        <is>
-          <t>Monitor</t>
+      <c r="K35" s="56" t="inlineStr">
+        <is>
+          <t>Act Now</t>
         </is>
       </c>
       <c r="L35" s="45" t="n">
@@ -3230,12 +3227,12 @@
       </c>
       <c r="H39" s="46" t="inlineStr">
         <is>
-          <t>New South Philadelphia A</t>
+          <t>Allegiant Stadium</t>
         </is>
       </c>
       <c r="I39" s="45" t="inlineStr">
         <is>
-          <t>NBA</t>
+          <t>NFL</t>
         </is>
       </c>
       <c r="J39" s="45" t="n">
@@ -3272,20 +3269,20 @@
       </c>
       <c r="H40" s="53" t="inlineStr">
         <is>
-          <t>New Dallas Arena</t>
+          <t>California Memorial Stad</t>
         </is>
       </c>
       <c r="I40" s="52" t="inlineStr">
         <is>
-          <t>NBA</t>
+          <t>NCAA</t>
         </is>
       </c>
       <c r="J40" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="K40" s="56" t="inlineStr">
-        <is>
-          <t>Act Now</t>
+      <c r="K40" s="51" t="inlineStr">
+        <is>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="L40" s="52" t="n">
@@ -3298,7 +3295,7 @@
       </c>
       <c r="N40" s="59" t="inlineStr">
         <is>
-          <t>✓  23 active projects (Act Now + Monitor) tracked.</t>
+          <t>✓  24 active projects (Act Now + Monitor) tracked.</t>
         </is>
       </c>
     </row>
@@ -3314,12 +3311,12 @@
       </c>
       <c r="H41" s="46" t="inlineStr">
         <is>
-          <t>Allegiant Stadium</t>
+          <t>Darrell K Royal–Texas Me</t>
         </is>
       </c>
       <c r="I41" s="45" t="inlineStr">
         <is>
-          <t>NFL</t>
+          <t>NCAA</t>
         </is>
       </c>
       <c r="J41" s="45" t="n">
@@ -13087,7 +13084,11 @@
         </is>
       </c>
       <c r="I199" s="64" t="inlineStr"/>
-      <c r="J199" s="64" t="inlineStr"/>
+      <c r="J199" s="64" t="inlineStr">
+        <is>
+          <t>Florida International University</t>
+        </is>
+      </c>
       <c r="K199" s="64" t="inlineStr"/>
     </row>
     <row r="200" ht="18" customHeight="1">
@@ -13545,7 +13546,11 @@
         </is>
       </c>
       <c r="I209" s="64" t="inlineStr"/>
-      <c r="J209" s="64" t="inlineStr"/>
+      <c r="J209" s="64" t="inlineStr">
+        <is>
+          <t>Eastern Michigan University</t>
+        </is>
+      </c>
       <c r="K209" s="64" t="inlineStr"/>
     </row>
     <row r="210" ht="18" customHeight="1">
@@ -13858,7 +13863,11 @@
         </is>
       </c>
       <c r="I216" s="62" t="inlineStr"/>
-      <c r="J216" s="62" t="inlineStr"/>
+      <c r="J216" s="62" t="inlineStr">
+        <is>
+          <t>Univ. of Tulsa Athletics</t>
+        </is>
+      </c>
       <c r="K216" s="62" t="inlineStr"/>
     </row>
     <row r="217" ht="18" customHeight="1">
@@ -14081,7 +14090,11 @@
         </is>
       </c>
       <c r="I221" s="64" t="inlineStr"/>
-      <c r="J221" s="64" t="inlineStr"/>
+      <c r="J221" s="64" t="inlineStr">
+        <is>
+          <t>University Athletic Association</t>
+        </is>
+      </c>
       <c r="K221" s="64" t="inlineStr"/>
     </row>
     <row r="222" ht="18" customHeight="1">
@@ -15980,7 +15993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S34"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16139,11 +16152,11 @@
         </is>
       </c>
       <c r="I2" s="67" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="J2" s="67" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>70%</t>
         </is>
       </c>
       <c r="K2" s="67" t="inlineStr">
@@ -16153,23 +16166,23 @@
       </c>
       <c r="L2" s="69" t="inlineStr">
         <is>
-          <t>The Chicago Bears are planning a new stadium with a capacity of 60,000, set for 2031. This project is still in the early stages of development.</t>
+          <t>There are discussions about the potential for a new stadium for the Chicago Bears in Northwest Indiana. Local officials are optimistic about the project's chances.</t>
         </is>
       </c>
       <c r="M2" s="69" t="inlineStr">
         <is>
-          <t>This new stadium project presents a significant opportunity for aluminum railings and structural components. Engaging early can position us favorably for future contracts.</t>
+          <t>A new stadium could significantly increase demand for aluminum railings and platforms. This project represents a major opportunity for our business in a high-profile venue.</t>
         </is>
       </c>
       <c r="N2" s="69" t="inlineStr">
         <is>
-          <t>The venue is planned for construction in 2031.</t>
+          <t>Local leaders believe the chances of securing a new stadium for the Bears have improved.</t>
         </is>
       </c>
       <c r="O2" s="69" t="inlineStr"/>
       <c r="P2" s="68" t="inlineStr">
         <is>
-          <t>https://www.si.com/nfl/bears/onsi/2-chicago-bears-contracts-that-will-age-poorly-during-2026-season</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNdmpZNzVGUnMwQmdYcGNaR0tIcEpiQ21EaWxHM0dWUU9sem9RS1VFemZYX05GODRha240dmlzWkRvc1psS3U5UmVFalpFWE5EdFAzaEtjWVU2VS1DbTQ0ZExHUWQ3NWxVNUJuV04xMjQxS2NwdXFaLWNLTnAxRFpVci1sbXltRnRWaTl2NUdxUXJzTEtWUTdDT1EzV1NNMnpWS0ZzcEJNLUZZaDJERThaSmNXSHJXWDZwM3BZLUpTaU1lZzM5bGpn?oc=5</t>
         </is>
       </c>
       <c r="Q2" s="70" t="inlineStr">
@@ -16186,69 +16199,69 @@
       </c>
       <c r="B3" s="63" t="inlineStr">
         <is>
-          <t>New South Philadelphia Arena</t>
+          <t>New Aloha Stadium</t>
         </is>
       </c>
       <c r="C3" s="64" t="inlineStr">
         <is>
-          <t>NBA</t>
+          <t>NCAA</t>
         </is>
       </c>
       <c r="D3" s="63" t="inlineStr">
         <is>
-          <t>Philadelphia 76ers</t>
+          <t>Hawaiʻi</t>
         </is>
       </c>
       <c r="E3" s="63" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="F3" s="64" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>HI</t>
         </is>
       </c>
       <c r="G3" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
+        <v>31000</v>
+      </c>
+      <c r="H3" s="71" t="inlineStr">
+        <is>
+          <t>Tier 3 — Design Phase</t>
         </is>
       </c>
       <c r="I3" s="64" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="J3" s="64" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="K3" s="64" t="inlineStr">
         <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L3" s="71" t="inlineStr">
-        <is>
-          <t>The Philadelphia 76ers are planning a new arena set to open in 2030. Discussions are ongoing about team improvements, but no specific details about the arena's construction are mentioned.</t>
-        </is>
-      </c>
-      <c r="M3" s="71" t="inlineStr">
-        <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a new sports venue. Engaging early could position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N3" s="71" t="inlineStr">
-        <is>
-          <t>The venue is confirmed as planned for the year 2030.</t>
-        </is>
-      </c>
-      <c r="O3" s="71" t="inlineStr"/>
+          <t>Major Renovation</t>
+        </is>
+      </c>
+      <c r="L3" s="72" t="inlineStr">
+        <is>
+          <t>Officials have held a blessing for the redevelopment of Aloha Stadium. This marks a significant milestone in the ongoing construction project.</t>
+        </is>
+      </c>
+      <c r="M3" s="72" t="inlineStr">
+        <is>
+          <t>This redevelopment is crucial for enhancing the venue's capacity and facilities, which can lead to increased demand for aluminum railings and platforms. Engaging in this project can position our company favorably in the market.</t>
+        </is>
+      </c>
+      <c r="N3" s="72" t="inlineStr">
+        <is>
+          <t>The article discusses a milestone in the redevelopment of Aloha Stadium.</t>
+        </is>
+      </c>
+      <c r="O3" s="72" t="inlineStr"/>
       <c r="P3" s="63" t="inlineStr">
         <is>
-          <t>https://heavy.com/sports/nba/philadelphia-76ers/urged-steer-clear-29-year-old-lakers-free-agent/</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQUEcxMTFNdEF4UE1iTURhNEhVamZEM1psVEJrWm1hYmFPSVlxcTVxVVRiUkc1SlgwS3BjTmVkVjdyLU4wclRpVUhiNWxPbzU5SlpwUzdRdU9jSV9UQTFidUI4enh3MnVUeGdNeHRpQmV4TDFRRXlsUGNORW5Sb281ck96eUNQS1MydTF3aHNfd3VpTngyNlFQZHB1c21CenEyU3l5eTZ0X1RPT1hDSDJZZG5n0gHGAUFVX3lxTFBCck91VGdNeGdXdzR0aE1LaVNaa0dQNHM1UUNLZkIzTGNrMTAwS3NWWjdPVmVoYlBSZEl6OTUydXNQZnZIclVINmZFcXd2SHBnUktNZmhMOFltZUxacklqd2pZWVVSTEdaNmpjcjVLcTk1R1FWbUZDTTlMdzNwOVdWUG1RMEZjUkFGSlVRVXhTWjNyem5pRkNFRklwZWFoZWpOLWg5RU9oRjRtaFNYSGdzVlp5dFNqaE5pNVd5Y29IQlFMeUduZw?oc=5</t>
         </is>
       </c>
       <c r="Q3" s="70" t="inlineStr">
@@ -16265,43 +16278,43 @@
       </c>
       <c r="B4" s="68" t="inlineStr">
         <is>
-          <t>New Dallas Arena</t>
+          <t>New Huntington Bank Field</t>
         </is>
       </c>
       <c r="C4" s="67" t="inlineStr">
         <is>
-          <t>NBA</t>
+          <t>NFL</t>
         </is>
       </c>
       <c r="D4" s="68" t="inlineStr">
         <is>
-          <t>Dallas Mavericks</t>
+          <t>Cleveland Browns</t>
         </is>
       </c>
       <c r="E4" s="68" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Brook Park</t>
         </is>
       </c>
       <c r="F4" s="67" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G4" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
+        <v>67500</v>
+      </c>
+      <c r="H4" s="73" t="inlineStr">
+        <is>
+          <t>Tier 4 — Procurement</t>
         </is>
       </c>
       <c r="I4" s="67" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="J4" s="67" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="K4" s="67" t="inlineStr">
@@ -16311,28 +16324,28 @@
       </c>
       <c r="L4" s="69" t="inlineStr">
         <is>
-          <t>The Dallas Mavericks are preparing for the 2026 NBA Draft. The new arena is planned for 2031, indicating future development.</t>
+          <t>Cleveland City Council is holding a special meeting about the lease for Huntington Bank Field. The venue is currently under construction.</t>
         </is>
       </c>
       <c r="M4" s="69" t="inlineStr">
         <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a new sports venue. Engaging early can position us favorably for future contracts.</t>
+          <t>This project is significant as it involves a major NFL venue, which could lead to substantial demand for aluminum railings and platforms. Engaging early can position us favorably for future contracts.</t>
         </is>
       </c>
       <c r="N4" s="69" t="inlineStr">
         <is>
-          <t>The venue is confirmed as planned for 2031.</t>
+          <t>Construction officially started on the new NFL stadium on April 30, 2026.</t>
         </is>
       </c>
       <c r="O4" s="69" t="inlineStr"/>
       <c r="P4" s="68" t="inlineStr">
         <is>
-          <t>https://www.si.com/nba/mavericks/onsi/monday-dallas-mavericks-mock-final-predictions-one-day-ahead-2026-nba-draft-</t>
-        </is>
-      </c>
-      <c r="Q4" s="65" t="inlineStr">
-        <is>
-          <t>engage_now</t>
+          <t>https://www.constructiondive.com/news/aecom-hunt-turner-jv-cleveland-browns-stadium-project/819230/</t>
+        </is>
+      </c>
+      <c r="Q4" s="73" t="inlineStr">
+        <is>
+          <t>too_late</t>
         </is>
       </c>
       <c r="R4" s="67" t="inlineStr"/>
@@ -16344,43 +16357,43 @@
       </c>
       <c r="B5" s="63" t="inlineStr">
         <is>
-          <t>New Spurs Arena</t>
+          <t>New Las Vegas Stadium†</t>
         </is>
       </c>
       <c r="C5" s="64" t="inlineStr">
         <is>
-          <t>NBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="D5" s="63" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Las Vegas Athletics</t>
         </is>
       </c>
       <c r="E5" s="63" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Paradise</t>
         </is>
       </c>
       <c r="F5" s="64" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="G5" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
+        <v>33000</v>
+      </c>
+      <c r="H5" s="73" t="inlineStr">
+        <is>
+          <t>Tier 4 — Procurement</t>
         </is>
       </c>
       <c r="I5" s="64" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="J5" s="64" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="K5" s="64" t="inlineStr">
@@ -16388,2325 +16401,34 @@
           <t>New Construction</t>
         </is>
       </c>
-      <c r="L5" s="71" t="inlineStr">
-        <is>
-          <t>The New Spurs Arena is planned for construction in 2032. This project is in the early stages of development.</t>
-        </is>
-      </c>
-      <c r="M5" s="71" t="inlineStr">
-        <is>
-          <t>This venue will require significant aluminum railings and platforms, presenting a key opportunity for our business. Engaging early can position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N5" s="71" t="inlineStr">
-        <is>
-          <t>The venue is confirmed as planned for 2032.</t>
-        </is>
-      </c>
-      <c r="O5" s="71" t="inlineStr"/>
+      <c r="L5" s="72" t="inlineStr">
+        <is>
+          <t>Funding has been secured for the construction of the Las Vegas Athletics' new ballpark. The project is currently under construction.</t>
+        </is>
+      </c>
+      <c r="M5" s="72" t="inlineStr">
+        <is>
+          <t>This project represents a significant opportunity for aluminum railings and platforms in a new sports venue. Secured funding indicates a commitment to proceed, which is crucial for our business.</t>
+        </is>
+      </c>
+      <c r="N5" s="72" t="inlineStr">
+        <is>
+          <t>Construction is underway with the lower bowl of the stadium taking shape.</t>
+        </is>
+      </c>
+      <c r="O5" s="72" t="inlineStr"/>
       <c r="P5" s="63" t="inlineStr">
         <is>
-          <t>https://www.si.com/nba/rockets/onsi/rockets-legend-with-some-hilarious-words-after-knicks-won-nba-finals</t>
-        </is>
-      </c>
-      <c r="Q5" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
+          <t>https://www.washingtonpost.com/sports/mlb/2026/05/21/athletics-as-stadium-vegas/8465de94-557d-11f1-9c40-7a0a12d9e745_story.html</t>
+        </is>
+      </c>
+      <c r="Q5" s="73" t="inlineStr">
+        <is>
+          <t>too_late</t>
         </is>
       </c>
       <c r="R5" s="64" t="inlineStr"/>
       <c r="S5" s="64" t="inlineStr"/>
-    </row>
-    <row r="6" ht="75" customHeight="1">
-      <c r="A6" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="68" t="inlineStr">
-        <is>
-          <t>New White Sox Stadium</t>
-        </is>
-      </c>
-      <c r="C6" s="67" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="D6" s="68" t="inlineStr">
-        <is>
-          <t>Chicago White Sox</t>
-        </is>
-      </c>
-      <c r="E6" s="68" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="F6" s="67" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="G6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I6" s="67" t="n">
-        <v>60</v>
-      </c>
-      <c r="J6" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K6" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L6" s="69" t="inlineStr">
-        <is>
-          <t>The Chicago White Sox are set to play a series against the Cleveland Guardians at Rate Field. This indicates ongoing activities at the venue.</t>
-        </is>
-      </c>
-      <c r="M6" s="69" t="inlineStr">
-        <is>
-          <t>This matters for our business as it highlights potential future construction needs for the new stadium. Engaging early could position us favorably for upcoming projects.</t>
-        </is>
-      </c>
-      <c r="N6" s="69" t="inlineStr">
-        <is>
-          <t>The article discusses the Chicago White Sox, indicating the venue is active.</t>
-        </is>
-      </c>
-      <c r="O6" s="69" t="inlineStr"/>
-      <c r="P6" s="68" t="inlineStr">
-        <is>
-          <t>https://www.greenbaypressgazette.com/story/sports/mlb/2026/06/22/guardians-at-white-sox-odds-picks-and-predictions/90639428007/</t>
-        </is>
-      </c>
-      <c r="Q6" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R6" s="67" t="inlineStr"/>
-      <c r="S6" s="67" t="inlineStr"/>
-    </row>
-    <row r="7" ht="75" customHeight="1">
-      <c r="A7" s="64" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="63" t="inlineStr">
-        <is>
-          <t>New Chiefs Stadium</t>
-        </is>
-      </c>
-      <c r="C7" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D7" s="63" t="inlineStr">
-        <is>
-          <t>Kansas City Chiefs</t>
-        </is>
-      </c>
-      <c r="E7" s="63" t="inlineStr">
-        <is>
-          <t>Kansas City</t>
-        </is>
-      </c>
-      <c r="F7" s="64" t="inlineStr">
-        <is>
-          <t>KS</t>
-        </is>
-      </c>
-      <c r="G7" s="64" t="n">
-        <v>65000</v>
-      </c>
-      <c r="H7" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I7" s="64" t="n">
-        <v>60</v>
-      </c>
-      <c r="J7" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K7" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L7" s="71" t="inlineStr">
-        <is>
-          <t>The New Chiefs Stadium is planned for construction in 2031. This project is confirmed as part of the Kansas City Chiefs' future developments.</t>
-        </is>
-      </c>
-      <c r="M7" s="71" t="inlineStr">
-        <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a large venue. Engaging early can position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N7" s="71" t="inlineStr">
-        <is>
-          <t>Funding for the Chiefs stadium deal was approved in December 2025.</t>
-        </is>
-      </c>
-      <c r="O7" s="71" t="inlineStr"/>
-      <c r="P7" s="63" t="inlineStr">
-        <is>
-          <t>https://www.axios.com/local/kansas-city/2026/01/21/stadiums-are-becoming-micro-cities</t>
-        </is>
-      </c>
-      <c r="Q7" s="65" t="inlineStr">
-        <is>
-          <t>engage_now</t>
-        </is>
-      </c>
-      <c r="R7" s="64" t="inlineStr"/>
-      <c r="S7" s="64" t="inlineStr"/>
-    </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="67" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="68" t="inlineStr">
-        <is>
-          <t>New Rays Stadium†</t>
-        </is>
-      </c>
-      <c r="C8" s="67" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="D8" s="68" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="E8" s="68" t="inlineStr">
-        <is>
-          <t>Tampa</t>
-        </is>
-      </c>
-      <c r="F8" s="67" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="G8" s="67" t="n">
-        <v>31000</v>
-      </c>
-      <c r="H8" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I8" s="67" t="n">
-        <v>49</v>
-      </c>
-      <c r="J8" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K8" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L8" s="69" t="inlineStr">
-        <is>
-          <t>The Tampa Bay Rays are planning a new stadium set to open in 2029. This project is still in the early stages of development.</t>
-        </is>
-      </c>
-      <c r="M8" s="69" t="inlineStr">
-        <is>
-          <t>This new stadium presents a significant opportunity for aluminum railings and structural components. Engaging early can position us favorably in the bidding process.</t>
-        </is>
-      </c>
-      <c r="N8" s="69" t="inlineStr">
-        <is>
-          <t>Funding for the $2.3 billion stadium has been tentatively approved by local officials.</t>
-        </is>
-      </c>
-      <c r="O8" s="69" t="inlineStr"/>
-      <c r="P8" s="68" t="inlineStr">
-        <is>
-          <t>https://bleacherreport.com/articles/25427989-rays-new-23b-stadium-tentatively-approved-local-officials-latest-timeline-revealed</t>
-        </is>
-      </c>
-      <c r="Q8" s="65" t="inlineStr">
-        <is>
-          <t>engage_now</t>
-        </is>
-      </c>
-      <c r="R8" s="67" t="inlineStr"/>
-      <c r="S8" s="67" t="inlineStr"/>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="64" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="63" t="inlineStr">
-        <is>
-          <t>New Royals Stadium</t>
-        </is>
-      </c>
-      <c r="C9" s="64" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="D9" s="63" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="E9" s="63" t="inlineStr">
-        <is>
-          <t>Kansas City</t>
-        </is>
-      </c>
-      <c r="F9" s="64" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="G9" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I9" s="64" t="n">
-        <v>47</v>
-      </c>
-      <c r="J9" s="64" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K9" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L9" s="71" t="inlineStr">
-        <is>
-          <t>The Kansas City Royals are planning a new stadium set to open in 2030. This project is still in the early stages of development.</t>
-        </is>
-      </c>
-      <c r="M9" s="71" t="inlineStr">
-        <is>
-          <t>A new stadium presents significant opportunities for aluminum railings and structural components. Engaging early can position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N9" s="71" t="inlineStr">
-        <is>
-          <t>Kansas City officials have proposed an ordinance for public funding towards the new stadium.</t>
-        </is>
-      </c>
-      <c r="O9" s="71" t="inlineStr"/>
-      <c r="P9" s="63" t="inlineStr">
-        <is>
-          <t>https://www.mlbtraderumors.com/2026/04/kansas-city-officials-propose-royals-stadium-plan.html</t>
-        </is>
-      </c>
-      <c r="Q9" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R9" s="64" t="inlineStr"/>
-      <c r="S9" s="64" t="inlineStr"/>
-    </row>
-    <row r="10" ht="75" customHeight="1">
-      <c r="A10" s="67" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="68" t="inlineStr">
-        <is>
-          <t>New Plano Arena</t>
-        </is>
-      </c>
-      <c r="C10" s="67" t="inlineStr">
-        <is>
-          <t>NHL</t>
-        </is>
-      </c>
-      <c r="D10" s="68" t="inlineStr">
-        <is>
-          <t>Dallas Stars</t>
-        </is>
-      </c>
-      <c r="E10" s="68" t="inlineStr">
-        <is>
-          <t>Plano</t>
-        </is>
-      </c>
-      <c r="F10" s="67" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="G10" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I10" s="67" t="n">
-        <v>47</v>
-      </c>
-      <c r="J10" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K10" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L10" s="69" t="inlineStr">
-        <is>
-          <t>The Ottawa Senators are attempting to acquire Jason Robertson from the Dallas Stars. This indicates ongoing team developments but does not directly relate to the venue's construction.</t>
-        </is>
-      </c>
-      <c r="M10" s="69" t="inlineStr">
-        <is>
-          <t>The acquisition of players can impact the team's performance and fan engagement, which may influence future venue developments. However, this article does not provide direct information about the venue's status.</t>
-        </is>
-      </c>
-      <c r="N10" s="69" t="inlineStr">
-        <is>
-          <t>Plano City Council approved a funding plan for the new arena.</t>
-        </is>
-      </c>
-      <c r="O10" s="69" t="inlineStr"/>
-      <c r="P10" s="68" t="inlineStr">
-        <is>
-          <t>https://www.espn.com/nhl/story/_/id/49005792/plano-approves-funding-plan-potential-dallas-stars-arena</t>
-        </is>
-      </c>
-      <c r="Q10" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R10" s="67" t="inlineStr"/>
-      <c r="S10" s="67" t="inlineStr"/>
-    </row>
-    <row r="11" ht="75" customHeight="1">
-      <c r="A11" s="64" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="63" t="inlineStr">
-        <is>
-          <t>New Broncos Stadium</t>
-        </is>
-      </c>
-      <c r="C11" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D11" s="63" t="inlineStr">
-        <is>
-          <t>Denver Broncos</t>
-        </is>
-      </c>
-      <c r="E11" s="63" t="inlineStr">
-        <is>
-          <t>Denver</t>
-        </is>
-      </c>
-      <c r="F11" s="64" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
-      <c r="G11" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I11" s="64" t="n">
-        <v>30</v>
-      </c>
-      <c r="J11" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K11" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L11" s="71" t="inlineStr">
-        <is>
-          <t>The Denver Broncos are planning a new stadium set for 2031. This project is still in the early stages of development.</t>
-        </is>
-      </c>
-      <c r="M11" s="71" t="inlineStr">
-        <is>
-          <t>A new stadium presents significant opportunities for aluminum railings and structural components. Engaging early can position us favorably in the bidding process.</t>
-        </is>
-      </c>
-      <c r="N11" s="71" t="inlineStr">
-        <is>
-          <t>Site construction is slated to start as early as next year.</t>
-        </is>
-      </c>
-      <c r="O11" s="71" t="inlineStr"/>
-      <c r="P11" s="63" t="inlineStr">
-        <is>
-          <t>https://www.axios.com/local/denver/2026/02/13/broncos-unveil-preliminary-framework-new-stadium</t>
-        </is>
-      </c>
-      <c r="Q11" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R11" s="64" t="inlineStr"/>
-      <c r="S11" s="64" t="inlineStr"/>
-    </row>
-    <row r="12" ht="75" customHeight="1">
-      <c r="A12" s="67" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="68" t="inlineStr">
-        <is>
-          <t>Future South Florida on-campus stadium</t>
-        </is>
-      </c>
-      <c r="C12" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D12" s="68" t="inlineStr">
-        <is>
-          <t>South Florida</t>
-        </is>
-      </c>
-      <c r="E12" s="68" t="inlineStr">
-        <is>
-          <t>Tampa</t>
-        </is>
-      </c>
-      <c r="F12" s="67" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="G12" s="67" t="n">
-        <v>35000</v>
-      </c>
-      <c r="H12" s="74" t="inlineStr">
-        <is>
-          <t>Tier 3 — Design Phase</t>
-        </is>
-      </c>
-      <c r="I12" s="67" t="n">
-        <v>30</v>
-      </c>
-      <c r="J12" s="67" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K12" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L12" s="69" t="inlineStr">
-        <is>
-          <t>A new on-campus stadium for South Florida is under construction. This project is expected to be completed by 2027.</t>
-        </is>
-      </c>
-      <c r="M12" s="69" t="inlineStr">
-        <is>
-          <t>The influx of wealth from tech IPOs could increase funding opportunities for sports venues. This may lead to more demand for aluminum railings and structural components.</t>
-        </is>
-      </c>
-      <c r="N12" s="69" t="inlineStr">
-        <is>
-          <t>The venue is currently under construction.</t>
-        </is>
-      </c>
-      <c r="O12" s="69" t="inlineStr"/>
-      <c r="P12" s="68" t="inlineStr">
-        <is>
-          <t>https://www.foxbusiness.com/real-estate/california-exodus-2-0-how-spacex-tech-ipos-could-trigger-next-massive-wealth-flight-florida</t>
-        </is>
-      </c>
-      <c r="Q12" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R12" s="67" t="inlineStr"/>
-      <c r="S12" s="67" t="inlineStr"/>
-    </row>
-    <row r="13" ht="75" customHeight="1">
-      <c r="A13" s="64" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="63" t="inlineStr">
-        <is>
-          <t>New Huntington Bank Field</t>
-        </is>
-      </c>
-      <c r="C13" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D13" s="63" t="inlineStr">
-        <is>
-          <t>Cleveland Browns</t>
-        </is>
-      </c>
-      <c r="E13" s="63" t="inlineStr">
-        <is>
-          <t>Brook Park</t>
-        </is>
-      </c>
-      <c r="F13" s="64" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="G13" s="64" t="n">
-        <v>67500</v>
-      </c>
-      <c r="H13" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I13" s="64" t="n">
-        <v>28</v>
-      </c>
-      <c r="J13" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K13" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L13" s="71" t="inlineStr">
-        <is>
-          <t>The New Huntington Bank Field is under construction as part of a new project for the Cleveland Browns. This venue is set to be completed by 2029.</t>
-        </is>
-      </c>
-      <c r="M13" s="71" t="inlineStr">
-        <is>
-          <t>This project represents a significant investment in a new sports venue, which could lead to increased demand for aluminum railings and platforms. Engaging early could position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N13" s="71" t="inlineStr">
-        <is>
-          <t>Construction has officially started as of April 30, 2026.</t>
-        </is>
-      </c>
-      <c r="O13" s="71" t="inlineStr"/>
-      <c r="P13" s="63" t="inlineStr">
-        <is>
-          <t>https://www.constructiondive.com/news/aecom-hunt-turner-jv-cleveland-browns-stadium-project/819230/</t>
-        </is>
-      </c>
-      <c r="Q13" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R13" s="64" t="inlineStr"/>
-      <c r="S13" s="64" t="inlineStr"/>
-    </row>
-    <row r="14" ht="75" customHeight="1">
-      <c r="A14" s="67" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="68" t="inlineStr">
-        <is>
-          <t>New Stadium at RFK Campus</t>
-        </is>
-      </c>
-      <c r="C14" s="67" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D14" s="68" t="inlineStr">
-        <is>
-          <t>Washington Commanders</t>
-        </is>
-      </c>
-      <c r="E14" s="68" t="inlineStr">
-        <is>
-          <t>Washington</t>
-        </is>
-      </c>
-      <c r="F14" s="67" t="inlineStr">
-        <is>
-          <t>DC</t>
-        </is>
-      </c>
-      <c r="G14" s="67" t="n">
-        <v>65000</v>
-      </c>
-      <c r="H14" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I14" s="67" t="n">
-        <v>28</v>
-      </c>
-      <c r="J14" s="67" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K14" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L14" s="69" t="inlineStr">
-        <is>
-          <t>The Washington Commanders' new stadium is under construction and set to open in 2030. The team is currently addressing its identity crisis as it prepares for the upcoming season.</t>
-        </is>
-      </c>
-      <c r="M14" s="69" t="inlineStr">
-        <is>
-          <t>This project represents a significant investment in a new venue, which could lead to increased demand for aluminum railings and structural components. Engaging early could position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N14" s="69" t="inlineStr">
-        <is>
-          <t>Groundbreaking is expected to start this year.</t>
-        </is>
-      </c>
-      <c r="O14" s="69" t="inlineStr"/>
-      <c r="P14" s="68" t="inlineStr">
-        <is>
-          <t>https://www.sportingnews.com/us/nfl/washington-commanders/news/commanders-released-photos-new-stadium-washington-dc-looks-incredible/cbfe130bc34f0a0c3a58a406</t>
-        </is>
-      </c>
-      <c r="Q14" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R14" s="67" t="inlineStr"/>
-      <c r="S14" s="67" t="inlineStr"/>
-    </row>
-    <row r="15" ht="75" customHeight="1">
-      <c r="A15" s="64" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="63" t="inlineStr">
-        <is>
-          <t>New Nissan Stadium</t>
-        </is>
-      </c>
-      <c r="C15" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D15" s="63" t="inlineStr">
-        <is>
-          <t>Tennessee Titans</t>
-        </is>
-      </c>
-      <c r="E15" s="63" t="inlineStr">
-        <is>
-          <t>Nashville</t>
-        </is>
-      </c>
-      <c r="F15" s="64" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="G15" s="64" t="n">
-        <v>60000</v>
-      </c>
-      <c r="H15" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I15" s="64" t="n">
-        <v>26</v>
-      </c>
-      <c r="J15" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K15" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L15" s="71" t="inlineStr">
-        <is>
-          <t>The New Nissan Stadium is under construction and set to be completed by 2027. The Tennessee Titans are preparing for the upcoming season with a new coaching staff and a young roster.</t>
-        </is>
-      </c>
-      <c r="M15" s="71" t="inlineStr">
-        <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a major sports venue. Engaging early can position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N15" s="71" t="inlineStr">
-        <is>
-          <t>Construction is on track for completion in February 2027.</t>
-        </is>
-      </c>
-      <c r="O15" s="71" t="inlineStr"/>
-      <c r="P15" s="63" t="inlineStr">
-        <is>
-          <t>https://www.greenwichtime.com/sports/article/tennessee-titans-new-enclosed-stadium-on-track-22094769.php</t>
-        </is>
-      </c>
-      <c r="Q15" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R15" s="64" t="inlineStr"/>
-      <c r="S15" s="64" t="inlineStr"/>
-    </row>
-    <row r="16" ht="75" customHeight="1">
-      <c r="A16" s="67" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="68" t="inlineStr">
-        <is>
-          <t>New Las Vegas Stadium†</t>
-        </is>
-      </c>
-      <c r="C16" s="67" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="D16" s="68" t="inlineStr">
-        <is>
-          <t>Las Vegas Athletics</t>
-        </is>
-      </c>
-      <c r="E16" s="68" t="inlineStr">
-        <is>
-          <t>Paradise</t>
-        </is>
-      </c>
-      <c r="F16" s="67" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="G16" s="67" t="n">
-        <v>33000</v>
-      </c>
-      <c r="H16" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I16" s="67" t="n">
-        <v>24</v>
-      </c>
-      <c r="J16" s="67" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K16" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L16" s="69" t="inlineStr">
-        <is>
-          <t>Funding has been secured for the construction of the new Las Vegas ballpark. The project is currently under construction.</t>
-        </is>
-      </c>
-      <c r="M16" s="69" t="inlineStr">
-        <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a new sports venue. Secured funding indicates a commitment to proceed, which is crucial for our business.</t>
-        </is>
-      </c>
-      <c r="N16" s="69" t="inlineStr">
-        <is>
-          <t>Construction is underway with the lower bowl of the stadium taking shape.</t>
-        </is>
-      </c>
-      <c r="O16" s="69" t="inlineStr"/>
-      <c r="P16" s="68" t="inlineStr">
-        <is>
-          <t>https://www.washingtonpost.com/sports/mlb/2026/05/21/athletics-as-stadium-vegas/8465de94-557d-11f1-9c40-7a0a12d9e745_story.html</t>
-        </is>
-      </c>
-      <c r="Q16" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R16" s="67" t="inlineStr"/>
-      <c r="S16" s="67" t="inlineStr"/>
-    </row>
-    <row r="17" ht="75" customHeight="1">
-      <c r="A17" s="64" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="63" t="inlineStr">
-        <is>
-          <t>New Aloha Stadium</t>
-        </is>
-      </c>
-      <c r="C17" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D17" s="63" t="inlineStr">
-        <is>
-          <t>Hawaiʻi</t>
-        </is>
-      </c>
-      <c r="E17" s="63" t="inlineStr">
-        <is>
-          <t>Honolulu</t>
-        </is>
-      </c>
-      <c r="F17" s="64" t="inlineStr">
-        <is>
-          <t>HI</t>
-        </is>
-      </c>
-      <c r="G17" s="64" t="n">
-        <v>31000</v>
-      </c>
-      <c r="H17" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I17" s="64" t="n">
-        <v>21</v>
-      </c>
-      <c r="J17" s="64" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K17" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L17" s="71" t="inlineStr">
-        <is>
-          <t>The New Aloha Stadium is currently under construction and is planned to be completed by 2029. This project is significant for the local community and sports events.</t>
-        </is>
-      </c>
-      <c r="M17" s="71" t="inlineStr">
-        <is>
-          <t>The construction of the stadium presents opportunities for aluminum railings and structural components. Engaging in this project could lead to substantial business growth.</t>
-        </is>
-      </c>
-      <c r="N17" s="71" t="inlineStr">
-        <is>
-          <t>Construction is currently underway, but there are complications with utility lines.</t>
-        </is>
-      </c>
-      <c r="O17" s="71" t="inlineStr"/>
-      <c r="P17" s="63" t="inlineStr">
-        <is>
-          <t>https://www.hawaiipublicradio.org/local-news/2026-04-17/tangled-utility-lines-complicate-aloha-stadium-project</t>
-        </is>
-      </c>
-      <c r="Q17" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R17" s="64" t="inlineStr"/>
-      <c r="S17" s="64" t="inlineStr"/>
-    </row>
-    <row r="18" ht="75" customHeight="1">
-      <c r="A18" s="67" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="68" t="inlineStr">
-        <is>
-          <t>Continental Coliseum</t>
-        </is>
-      </c>
-      <c r="C18" s="67" t="inlineStr">
-        <is>
-          <t>NBA</t>
-        </is>
-      </c>
-      <c r="D18" s="68" t="inlineStr">
-        <is>
-          <t>Oklahoma City Thunder</t>
-        </is>
-      </c>
-      <c r="E18" s="68" t="inlineStr">
-        <is>
-          <t>Oklahoma City</t>
-        </is>
-      </c>
-      <c r="F18" s="67" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G18" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I18" s="67" t="n">
-        <v>19</v>
-      </c>
-      <c r="J18" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K18" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L18" s="69" t="inlineStr">
-        <is>
-          <t>The Oklahoma City Thunder's new venue, Continental Coliseum, is currently under construction. The project is set to be completed by 2028.</t>
-        </is>
-      </c>
-      <c r="M18" s="69" t="inlineStr">
-        <is>
-          <t>This new construction presents an opportunity for aluminum railings and platforms. Engaging in this project could lead to significant business for our company.</t>
-        </is>
-      </c>
-      <c r="N18" s="69" t="inlineStr">
-        <is>
-          <t>Construction has officially started on the Continental Coliseum.</t>
-        </is>
-      </c>
-      <c r="O18" s="69" t="inlineStr"/>
-      <c r="P18" s="68" t="inlineStr">
-        <is>
-          <t>https://www.constructiondive.com/news/flintco-mortenson-jv-breaks-ground-oklahoma-arena/816027/</t>
-        </is>
-      </c>
-      <c r="Q18" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R18" s="67" t="inlineStr"/>
-      <c r="S18" s="67" t="inlineStr"/>
-    </row>
-    <row r="19" ht="75" customHeight="1">
-      <c r="A19" s="64" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="63" t="inlineStr">
-        <is>
-          <t>Williams–Brice Stadium</t>
-        </is>
-      </c>
-      <c r="C19" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D19" s="63" t="inlineStr">
-        <is>
-          <t>South Carolina</t>
-        </is>
-      </c>
-      <c r="E19" s="63" t="inlineStr">
-        <is>
-          <t>Columbia</t>
-        </is>
-      </c>
-      <c r="F19" s="64" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="G19" s="64" t="n">
-        <v>77559</v>
-      </c>
-      <c r="H19" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I19" s="64" t="n">
-        <v>70</v>
-      </c>
-      <c r="J19" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K19" s="64" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L19" s="71" t="inlineStr">
-        <is>
-          <t>South Carolina athletics is considering a significant modernization project for Williams-Brice Stadium. This initiative aims to enhance the venue's facilities and overall experience.</t>
-        </is>
-      </c>
-      <c r="M19" s="71" t="inlineStr">
-        <is>
-          <t>This project could lead to increased demand for aluminum railings and platforms as part of the renovation. Engaging early could position us favorably in the bidding process.</t>
-        </is>
-      </c>
-      <c r="N19" s="71" t="inlineStr">
-        <is>
-          <t>The article discusses a billion-dollar modernization project for Williams-Brice Stadium.</t>
-        </is>
-      </c>
-      <c r="O19" s="71" t="inlineStr"/>
-      <c r="P19" s="63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQbm5PMW5IUTJUWllDMTJBX2xlWTk3bFVzU0Z1MEdnc005bDE0MjhwYVZZQXQ1RFZaUl9ZVmdEOXd2YWtNYUkydVJRRnpuY1BxVkVpUFFvbjVsdV9aSzBXNk1ZaWktc3FrTnBzaHExVU16MG5aLURlRGRhMGVHWjZDdFpFamx5MXc1MVV3Sl9xUFZQUzRielppeXVXY2JwaGJHT1dfV3BBcVRKVzN5RFBVdFA0Q3Jmbm4xY0ZiWHNLMUp2eFJoUEFXNWVCVDE1bzUyMUQwZVRscw?oc=5</t>
-        </is>
-      </c>
-      <c r="Q19" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R19" s="64" t="inlineStr"/>
-      <c r="S19" s="64" t="inlineStr"/>
-    </row>
-    <row r="20" ht="75" customHeight="1">
-      <c r="A20" s="67" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="68" t="inlineStr">
-        <is>
-          <t>Kyle Field</t>
-        </is>
-      </c>
-      <c r="C20" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D20" s="68" t="inlineStr">
-        <is>
-          <t>Texas A&amp;M</t>
-        </is>
-      </c>
-      <c r="E20" s="68" t="inlineStr">
-        <is>
-          <t>College Station</t>
-        </is>
-      </c>
-      <c r="F20" s="67" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="G20" s="67" t="n">
-        <v>102733</v>
-      </c>
-      <c r="H20" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I20" s="67" t="n">
-        <v>70</v>
-      </c>
-      <c r="J20" s="67" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K20" s="67" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L20" s="69" t="inlineStr">
-        <is>
-          <t>Kyle Field is set for redevelopment following approval from the Texas A&amp;M Board of Regents. This project aims to enhance the venue's facilities and overall experience.</t>
-        </is>
-      </c>
-      <c r="M20" s="69" t="inlineStr">
-        <is>
-          <t>The redevelopment of Kyle Field presents a significant opportunity for our aluminum railings and structural components. Enhancements to such a large venue can lead to substantial orders for our products.</t>
-        </is>
-      </c>
-      <c r="N20" s="69" t="inlineStr">
-        <is>
-          <t>The Texas A&amp;M Board of Regents has approved the redevelopment of Kyle Field.</t>
-        </is>
-      </c>
-      <c r="O20" s="69" t="inlineStr"/>
-      <c r="P20" s="68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE1MR0VKdUhndE5KSHIzV2phck9RYWJ0LUVCR0xIZklDQU1CaGY1c2ZWWHVqQklGNUNCVmVuSHBCNDdGWFBzS0JCZk1HRU0zMHNDOWNkUmdR?oc=5</t>
-        </is>
-      </c>
-      <c r="Q20" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R20" s="67" t="inlineStr"/>
-      <c r="S20" s="67" t="inlineStr"/>
-    </row>
-    <row r="21" ht="75" customHeight="1">
-      <c r="A21" s="64" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="63" t="inlineStr">
-        <is>
-          <t>Neyland Stadium</t>
-        </is>
-      </c>
-      <c r="C21" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D21" s="63" t="inlineStr">
-        <is>
-          <t>Tennessee</t>
-        </is>
-      </c>
-      <c r="E21" s="63" t="inlineStr">
-        <is>
-          <t>Knoxville</t>
-        </is>
-      </c>
-      <c r="F21" s="64" t="inlineStr">
-        <is>
-          <t>TN</t>
-        </is>
-      </c>
-      <c r="G21" s="64" t="n">
-        <v>101915</v>
-      </c>
-      <c r="H21" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I21" s="64" t="n">
-        <v>70</v>
-      </c>
-      <c r="J21" s="64" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K21" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L21" s="71" t="inlineStr">
-        <is>
-          <t>Construction for the Neyland Stadium Entertainment District is expected to start this summer. This project aims to enhance the venue's surrounding area.</t>
-        </is>
-      </c>
-      <c r="M21" s="71" t="inlineStr">
-        <is>
-          <t>This development could increase foot traffic and enhance the overall experience for fans, potentially leading to increased demand for aluminum railings and platforms.</t>
-        </is>
-      </c>
-      <c r="N21" s="71" t="inlineStr">
-        <is>
-          <t>The article discusses the construction of the Neyland Stadium Entertainment District.</t>
-        </is>
-      </c>
-      <c r="O21" s="71" t="inlineStr"/>
-      <c r="P21" s="63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNWDBoYWtISDBxQ2JrSnN3YWhjT1lvU0hhSnNzRHNyU2Q5clJja1ZtQ3FUSm40U29Da1FEaThOM2pkcmQ3MVdsVW5WNExuX1JHYlBxdV9pWkwtcVNaMkdNUUtqUkhYbFRSNTVjcFJVcVotWmNKNjBPUzhSTklsLWV3QmNnTDdpa0h1VjVMeWRHZUxoYWg2VGU5ZzdCcDBFM2F3V0FMYlRidDRVdHpx?oc=5</t>
-        </is>
-      </c>
-      <c r="Q21" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R21" s="64" t="inlineStr"/>
-      <c r="S21" s="64" t="inlineStr"/>
-    </row>
-    <row r="22" ht="75" customHeight="1">
-      <c r="A22" s="67" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="68" t="inlineStr">
-        <is>
-          <t>Tiger Stadium</t>
-        </is>
-      </c>
-      <c r="C22" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D22" s="68" t="inlineStr">
-        <is>
-          <t>LSU</t>
-        </is>
-      </c>
-      <c r="E22" s="68" t="inlineStr">
-        <is>
-          <t>Baton Rouge</t>
-        </is>
-      </c>
-      <c r="F22" s="67" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="G22" s="67" t="n">
-        <v>102321</v>
-      </c>
-      <c r="H22" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I22" s="67" t="n">
-        <v>70</v>
-      </c>
-      <c r="J22" s="67" t="inlineStr">
-        <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="K22" s="67" t="inlineStr">
-        <is>
-          <t>Expansion</t>
-        </is>
-      </c>
-      <c r="L22" s="69" t="inlineStr">
-        <is>
-          <t>LSU Athletics is proposing an expansion for Tiger Stadium. This could lead to significant upgrades and increased capacity.</t>
-        </is>
-      </c>
-      <c r="M22" s="69" t="inlineStr">
-        <is>
-          <t>An expansion project could enhance the stadium's facilities and attract more events, benefiting our aluminum railing and platform business.</t>
-        </is>
-      </c>
-      <c r="N22" s="69" t="inlineStr">
-        <is>
-          <t>The article discusses a proposal for expanding Tiger Stadium.</t>
-        </is>
-      </c>
-      <c r="O22" s="69" t="inlineStr"/>
-      <c r="P22" s="68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE51UDZTTWZ4bE9Ua1JwVnEyZjNqdnpleUVoUVRHUEdxdTNoX3dBSl9aUHZ4VjRzY3BpR1BuZDRZbnYwSUxGaGtVc2pWQ2hDemFERWRwZTdwQml2ODdEMksw?oc=5</t>
-        </is>
-      </c>
-      <c r="Q22" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R22" s="67" t="inlineStr"/>
-      <c r="S22" s="67" t="inlineStr"/>
-    </row>
-    <row r="23" ht="75" customHeight="1">
-      <c r="A23" s="64" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="63" t="inlineStr">
-        <is>
-          <t>Allegiant Stadium</t>
-        </is>
-      </c>
-      <c r="C23" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D23" s="63" t="inlineStr">
-        <is>
-          <t>Las Vegas Raiders</t>
-        </is>
-      </c>
-      <c r="E23" s="63" t="inlineStr">
-        <is>
-          <t>Paradise</t>
-        </is>
-      </c>
-      <c r="F23" s="64" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="G23" s="64" t="n">
-        <v>66000</v>
-      </c>
-      <c r="H23" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I23" s="64" t="n">
-        <v>60</v>
-      </c>
-      <c r="J23" s="64" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K23" s="64" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L23" s="71" t="inlineStr">
-        <is>
-          <t>The county is dipping into its reserve fund to make a bond payment for Allegiant Stadium. This indicates financial management issues related to the venue.</t>
-        </is>
-      </c>
-      <c r="M23" s="71" t="inlineStr">
-        <is>
-          <t>This situation may lead to future renovations or upgrades, impacting our aluminum railing and platform business. Monitoring financial stability is crucial for potential opportunities.</t>
-        </is>
-      </c>
-      <c r="N23" s="71" t="inlineStr">
-        <is>
-          <t>The county is using reserve funds to cover a bond payment for Allegiant Stadium.</t>
-        </is>
-      </c>
-      <c r="O23" s="71" t="inlineStr"/>
-      <c r="P23" s="63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPTmxSUi1OZEl0QXUtXzVGeHZacV9ILTRhbTZlNVI0dzV2U00ya2ZySlZaa21DemsxbUNibnpNRi1sU3NYYWxKc2tHSzJtSkFFbklCU0dOOXMtdjFVN0NnMDFqNnFLV29jeEtOMEhrdVVzZ0Fid05keXhUWGQ2Q1JPRlhzQWhDa2NTa3B2cmZoQS1jRTdydFNLQTBpem1WQUVoUkpnbXkxWGJuSzRnY1l6WnB5T0NXY1lHaFR1QVFJWGJvZw?oc=5</t>
-        </is>
-      </c>
-      <c r="Q23" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R23" s="64" t="inlineStr"/>
-      <c r="S23" s="64" t="inlineStr"/>
-    </row>
-    <row r="24" ht="75" customHeight="1">
-      <c r="A24" s="67" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="68" t="inlineStr">
-        <is>
-          <t>California Memorial Stadium</t>
-        </is>
-      </c>
-      <c r="C24" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D24" s="68" t="inlineStr">
-        <is>
-          <t>California</t>
-        </is>
-      </c>
-      <c r="E24" s="68" t="inlineStr">
-        <is>
-          <t>Berkeley</t>
-        </is>
-      </c>
-      <c r="F24" s="67" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="G24" s="67" t="n">
-        <v>62467</v>
-      </c>
-      <c r="H24" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I24" s="67" t="n">
-        <v>60</v>
-      </c>
-      <c r="J24" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K24" s="67" t="inlineStr">
-        <is>
-          <t>Minor Upgrade</t>
-        </is>
-      </c>
-      <c r="L24" s="69" t="inlineStr">
-        <is>
-          <t>FTX has purchased the naming rights to the field at California Memorial Stadium. This indicates a potential investment in the venue's branding.</t>
-        </is>
-      </c>
-      <c r="M24" s="69" t="inlineStr">
-        <is>
-          <t>This investment could lead to further enhancements or renovations at the stadium, which may require our aluminum products. Securing naming rights often precedes additional upgrades.</t>
-        </is>
-      </c>
-      <c r="N24" s="69" t="inlineStr">
-        <is>
-          <t>The article discusses FTX acquiring naming rights specifically for the field at California Memorial Stadium.</t>
-        </is>
-      </c>
-      <c r="O24" s="69" t="inlineStr"/>
-      <c r="P24" s="68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNbjY2LVA5N190cVF3RWQ2b1dMcW01cE5hbnZHWi1IVnd3UXp4RGNfUjdJS3RtOWQyaWo1dFBfdm1zcE1GMUFMT3RXU3BvOWhQX3pZbDZrOHV6S0l2Qm1KV3BEUjhCdWVrem9QZHZJRmtnWUlURjZvVkxmM1BiN1czd3RHX0RYMkhuNW55WHRKQUFtVTBOV29aLQ?oc=5</t>
-        </is>
-      </c>
-      <c r="Q24" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R24" s="67" t="inlineStr"/>
-      <c r="S24" s="67" t="inlineStr"/>
-    </row>
-    <row r="25" ht="75" customHeight="1">
-      <c r="A25" s="64" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="63" t="inlineStr">
-        <is>
-          <t>Darrell K Royal–Texas Memorial Stadium</t>
-        </is>
-      </c>
-      <c r="C25" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D25" s="63" t="inlineStr">
-        <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="E25" s="63" t="inlineStr">
-        <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="F25" s="64" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="G25" s="64" t="n">
-        <v>100119</v>
-      </c>
-      <c r="H25" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I25" s="64" t="n">
-        <v>60</v>
-      </c>
-      <c r="J25" s="64" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="K25" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L25" s="71" t="inlineStr">
-        <is>
-          <t>The article features photos of Texas Longhorns WR Isaiah Bond. It highlights his career but does not mention any construction or renovation plans.</t>
-        </is>
-      </c>
-      <c r="M25" s="71" t="inlineStr">
-        <is>
-          <t>This matters as it indicates ongoing interest in the team and venue, which could lead to future projects. Engaging with the venue could position us for upcoming opportunities.</t>
-        </is>
-      </c>
-      <c r="N25" s="71" t="inlineStr">
-        <is>
-          <t>The article is about the Texas Longhorns, which plays at the stadium.</t>
-        </is>
-      </c>
-      <c r="O25" s="71" t="inlineStr"/>
-      <c r="P25" s="63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPc05qN19sWUtIYThKczRJY2lrbS1VN2htdnRQQk9LUHd0b1RtYWNMNC1wVHZKbk95NlVLQ0pvbm1yMjVHSVJpbWtGXzJCVnNoUFUzM3p6TW8yNEowSWstc0t0UTRPUVlpcWtIVEg4SjctWGlmLVBOQ0xHdUtqVFdhZ0ZQX0ZMTDdyMTlLWnY4S0N5VHUxUDU3dEZkc3VrN29iclgtN3JLdU9BNkZ5MUsxTFdpWVQ2cGtkN25MX3hmRGdHMWV2eEMtTm1UT2cwS1lLOWRr?oc=5</t>
-        </is>
-      </c>
-      <c r="Q25" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R25" s="64" t="inlineStr"/>
-      <c r="S25" s="64" t="inlineStr"/>
-    </row>
-    <row r="26" ht="75" customHeight="1">
-      <c r="A26" s="67" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="68" t="inlineStr">
-        <is>
-          <t>Notre Dame Stadium</t>
-        </is>
-      </c>
-      <c r="C26" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D26" s="68" t="inlineStr">
-        <is>
-          <t>Notre Dame</t>
-        </is>
-      </c>
-      <c r="E26" s="68" t="inlineStr">
-        <is>
-          <t>Notre Dame</t>
-        </is>
-      </c>
-      <c r="F26" s="67" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G26" s="67" t="n">
-        <v>77622</v>
-      </c>
-      <c r="H26" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I26" s="67" t="n">
-        <v>60</v>
-      </c>
-      <c r="J26" s="67" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="K26" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L26" s="69" t="inlineStr">
-        <is>
-          <t>The article discusses a player from Notre Dame, suggesting engagement with the team and venue. However, it does not provide specific information about construction or renovations.</t>
-        </is>
-      </c>
-      <c r="M26" s="69" t="inlineStr">
-        <is>
-          <t>This matters as it indicates potential future developments or renovations at the venue. Engaging with the team could lead to opportunities for aluminum railings and platforms.</t>
-        </is>
-      </c>
-      <c r="N26" s="69" t="inlineStr">
-        <is>
-          <t>The article is about Notre Dame's football player, indicating ongoing activities related to the venue.</t>
-        </is>
-      </c>
-      <c r="O26" s="69" t="inlineStr"/>
-      <c r="P26" s="68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNVWVkZGVYdl8tbXZOZ0p3d3hrdnFHX2l5eHJwb1dGR0drek9jaW5US25XM1JxU29qRDBlVmRjZ0lyTTFRa0ZSby1BT3hFSmZVZzJmZXFjTGc2TTR5MzJ6NVV3WXNLVjRWRy1Rd1BNODI4a0UzSnR5aDlsRm5BRXZhRzJ4azk2Y1Q4VGFyR3B0STVjLXRZUnBfZk50S0xrd1hwdFRSTkppYm9VSGZ5WHc?oc=5</t>
-        </is>
-      </c>
-      <c r="Q26" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R26" s="67" t="inlineStr"/>
-      <c r="S26" s="67" t="inlineStr"/>
-    </row>
-    <row r="27" ht="75" customHeight="1">
-      <c r="A27" s="64" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="63" t="inlineStr">
-        <is>
-          <t>Sanford Stadium</t>
-        </is>
-      </c>
-      <c r="C27" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D27" s="63" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="E27" s="63" t="inlineStr">
-        <is>
-          <t>Athens</t>
-        </is>
-      </c>
-      <c r="F27" s="64" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="G27" s="64" t="n">
-        <v>93033</v>
-      </c>
-      <c r="H27" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I27" s="64" t="n">
-        <v>63</v>
-      </c>
-      <c r="J27" s="64" t="inlineStr">
-        <is>
-          <t>75%</t>
-        </is>
-      </c>
-      <c r="K27" s="64" t="inlineStr">
-        <is>
-          <t>Expansion</t>
-        </is>
-      </c>
-      <c r="L27" s="71" t="inlineStr">
-        <is>
-          <t>The Georgia football complex is set to undergo an expansion with more than $50 million in funding approved. This project will enhance the facilities for the Georgia football team.</t>
-        </is>
-      </c>
-      <c r="M27" s="71" t="inlineStr">
-        <is>
-          <t>This expansion is significant as it indicates investment in sports infrastructure, which could lead to increased demand for aluminum railings and platforms. Engaging in this project could position us favorably within the sports venue market.</t>
-        </is>
-      </c>
-      <c r="N27" s="71" t="inlineStr">
-        <is>
-          <t>Funding of over $50 million has been approved for the expansion of the Georgia football complex.</t>
-        </is>
-      </c>
-      <c r="O27" s="71" t="inlineStr"/>
-      <c r="P27" s="63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPMUU3S1AxVTl5bUJsQm0yU0FjaWRqNlFOM01jOG9CMjlJWElDeTRzWHc3ZWJDcHY0WGUyQnBLUnc3Qlpab29pd3dra2NGSFlESWZERnpPeWE4S05FdHhxVnR0aDVMTkl2X1JTejJaRWFtVFJZXzRvRU5fR0xTbFp5SG9JcTZKYUNWOXZZUDRCN3V4aHdsWFRTN2xxUzdob2NGN28taVR4d3pPeGhQdllfc1U3Qld5dEpOamt4M1dRU3puZGNaRXpQWlVNNWhlUC1CYWZlVWhR?oc=5</t>
-        </is>
-      </c>
-      <c r="Q27" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R27" s="64" t="inlineStr"/>
-      <c r="S27" s="64" t="inlineStr"/>
-    </row>
-    <row r="28" ht="75" customHeight="1">
-      <c r="A28" s="67" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="68" t="inlineStr">
-        <is>
-          <t>Jack Trice Stadium</t>
-        </is>
-      </c>
-      <c r="C28" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D28" s="68" t="inlineStr">
-        <is>
-          <t>Iowa State</t>
-        </is>
-      </c>
-      <c r="E28" s="68" t="inlineStr">
-        <is>
-          <t>Ames</t>
-        </is>
-      </c>
-      <c r="F28" s="67" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="G28" s="67" t="n">
-        <v>61500</v>
-      </c>
-      <c r="H28" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I28" s="67" t="n">
-        <v>53</v>
-      </c>
-      <c r="J28" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K28" s="67" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L28" s="69" t="inlineStr">
-        <is>
-          <t>Iowa State has agreed to allocate revenue from CYTown towards renovations at the Iowa State Center. Property tax implications are still being discussed.</t>
-        </is>
-      </c>
-      <c r="M28" s="69" t="inlineStr">
-        <is>
-          <t>This funding commitment could lead to significant renovations, impacting the venue's infrastructure. Improved facilities may enhance the overall experience for fans and athletes.</t>
-        </is>
-      </c>
-      <c r="N28" s="69" t="inlineStr">
-        <is>
-          <t>The article discusses funding for renovations at Iowa State Center.</t>
-        </is>
-      </c>
-      <c r="O28" s="69" t="inlineStr"/>
-      <c r="P28" s="68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNSnZrOFZZeWhOQThLRng1X1hGaU1NS0JRZmUwdVlCYmV1WnU2a0RMOW5ydUoyME4zektSTXpDM3d3V055M3pPVmVvTEw0Nkp2OFRmZWpJNXJLc05nOG1TU2tkZnNIczYxNy0xcFc2Ry1XQ3ZTRkdYQU1waUxxd2s4ckhYRnV2SGVseU05WEpuUjZjb1J5ZVZicU1FcWtZZXJUYWwwWkpSYXlPRVBoZDBGT1puOVQ3SlBMZmxjTFRzRVJFVmhUeGxNMFBHbmtGSWxkc0NQcHE1R0NzZw?oc=5</t>
-        </is>
-      </c>
-      <c r="Q28" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R28" s="67" t="inlineStr"/>
-      <c r="S28" s="67" t="inlineStr"/>
-    </row>
-    <row r="29" ht="75" customHeight="1">
-      <c r="A29" s="64" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="63" t="inlineStr">
-        <is>
-          <t>Pat Dye Field at Jordan–Hare Stadium</t>
-        </is>
-      </c>
-      <c r="C29" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D29" s="63" t="inlineStr">
-        <is>
-          <t>Auburn</t>
-        </is>
-      </c>
-      <c r="E29" s="63" t="inlineStr">
-        <is>
-          <t>Auburn</t>
-        </is>
-      </c>
-      <c r="F29" s="64" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="G29" s="64" t="n">
-        <v>88043</v>
-      </c>
-      <c r="H29" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I29" s="64" t="n">
-        <v>28</v>
-      </c>
-      <c r="J29" s="64" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="K29" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L29" s="71" t="inlineStr">
-        <is>
-          <t>The article reveals the contract details for Auburn's athletics director. This could indicate potential changes or developments in the athletics program.</t>
-        </is>
-      </c>
-      <c r="M29" s="71" t="inlineStr">
-        <is>
-          <t>Changes in leadership can impact future projects and funding for venue improvements. Staying informed on these developments is crucial for our business.</t>
-        </is>
-      </c>
-      <c r="N29" s="71" t="inlineStr">
-        <is>
-          <t>The Auburn Board of Trustees has granted final approval for the Jordan-Hare North Project.</t>
-        </is>
-      </c>
-      <c r="O29" s="71" t="inlineStr"/>
-      <c r="P29" s="63" t="inlineStr">
-        <is>
-          <t>https://auburntigers.com/news/2026/4/17/auburn-board-of-trustees-approves-jordan-hare-stadium-north-project</t>
-        </is>
-      </c>
-      <c r="Q29" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R29" s="64" t="inlineStr"/>
-      <c r="S29" s="64" t="inlineStr"/>
-    </row>
-    <row r="30" ht="75" customHeight="1">
-      <c r="A30" s="67" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="68" t="inlineStr">
-        <is>
-          <t>Gaylord Family Oklahoma Memorial Stadium</t>
-        </is>
-      </c>
-      <c r="C30" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D30" s="68" t="inlineStr">
-        <is>
-          <t>Oklahoma</t>
-        </is>
-      </c>
-      <c r="E30" s="68" t="inlineStr">
-        <is>
-          <t>Norman</t>
-        </is>
-      </c>
-      <c r="F30" s="67" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G30" s="67" t="n">
-        <v>80126</v>
-      </c>
-      <c r="H30" s="74" t="inlineStr">
-        <is>
-          <t>Tier 3 — Design Phase</t>
-        </is>
-      </c>
-      <c r="I30" s="67" t="n">
-        <v>30</v>
-      </c>
-      <c r="J30" s="67" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K30" s="67" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L30" s="69" t="inlineStr">
-        <is>
-          <t>The next phase of renovations for Gaylord Family Oklahoma Memorial Stadium has been approved. This indicates that the project is moving forward into the design phase.</t>
-        </is>
-      </c>
-      <c r="M30" s="69" t="inlineStr">
-        <is>
-          <t>This renovation presents an opportunity for our aluminum railings and structural components to be utilized in a major sports venue. Engaging in this project could enhance our visibility and reputation in the sports construction market.</t>
-        </is>
-      </c>
-      <c r="N30" s="69" t="inlineStr">
-        <is>
-          <t>The OU Board of Regents has approved the next phase of renovations for the stadium.</t>
-        </is>
-      </c>
-      <c r="O30" s="69" t="inlineStr"/>
-      <c r="P30" s="68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxQQ3ZoaERSZmJXLVFiWVJuYW1OaGJGd0szQ2ZSYjdhNlZuYnRqUzl4Yzk1ODJha09pS3FVX3NwRmVvclUxUFlKa0xvUEV3Z2tvS0Q4dEx1VG82V0cwV25qekVOdFdJVV9GcWM4UVpVZXVwMS1qTXA4Y056aWJNTi1DRG9DY3Z0UlUyMjR4SHNCZ1JDVDdOeXVRVmtYQUhEZUV5Q1Y0ZFo5TlZzbThwTFJPR0dWNkwyX05nRE4tbFRpYU9VYUQzZDVxb3dSek04VDg1RzVBUExVSQ?oc=5</t>
-        </is>
-      </c>
-      <c r="Q30" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R30" s="67" t="inlineStr"/>
-      <c r="S30" s="67" t="inlineStr"/>
-    </row>
-    <row r="31" ht="75" customHeight="1">
-      <c r="A31" s="64" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="63" t="inlineStr">
-        <is>
-          <t>Spartan Stadium</t>
-        </is>
-      </c>
-      <c r="C31" s="64" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D31" s="63" t="inlineStr">
-        <is>
-          <t>Michigan State</t>
-        </is>
-      </c>
-      <c r="E31" s="63" t="inlineStr">
-        <is>
-          <t>East Lansing</t>
-        </is>
-      </c>
-      <c r="F31" s="64" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
-      <c r="G31" s="64" t="n">
-        <v>74866</v>
-      </c>
-      <c r="H31" s="74" t="inlineStr">
-        <is>
-          <t>Tier 3 — Design Phase</t>
-        </is>
-      </c>
-      <c r="I31" s="64" t="n">
-        <v>28</v>
-      </c>
-      <c r="J31" s="64" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K31" s="64" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L31" s="71" t="inlineStr">
-        <is>
-          <t>Michigan State has set a significant fundraising goal to enhance its athletic facilities. This initiative indicates a commitment to improving the venue's infrastructure.</t>
-        </is>
-      </c>
-      <c r="M31" s="71" t="inlineStr">
-        <is>
-          <t>Upgrades to athletic facilities can lead to increased attendance and revenue, directly impacting the demand for aluminum railings and platforms. Engaging in this project could position us favorably in the bidding process.</t>
-        </is>
-      </c>
-      <c r="N31" s="71" t="inlineStr">
-        <is>
-          <t>Michigan State is working with architects and a construction group for the Spartan Stadium renovations.</t>
-        </is>
-      </c>
-      <c r="O31" s="71" t="inlineStr"/>
-      <c r="P31" s="63" t="inlineStr">
-        <is>
-          <t>https://www.si.com/college/michiganstate/spartans-batt-eyeing-several-stadium-transformations</t>
-        </is>
-      </c>
-      <c r="Q31" s="70" t="inlineStr">
-        <is>
-          <t>monitor</t>
-        </is>
-      </c>
-      <c r="R31" s="64" t="inlineStr"/>
-      <c r="S31" s="64" t="inlineStr"/>
-    </row>
-    <row r="32" ht="75" customHeight="1">
-      <c r="A32" s="67" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="68" t="inlineStr">
-        <is>
-          <t>Empower Field at Mile High</t>
-        </is>
-      </c>
-      <c r="C32" s="67" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D32" s="68" t="inlineStr">
-        <is>
-          <t>Denver Broncos</t>
-        </is>
-      </c>
-      <c r="E32" s="68" t="inlineStr">
-        <is>
-          <t>Denver</t>
-        </is>
-      </c>
-      <c r="F32" s="67" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
-      <c r="G32" s="67" t="n">
-        <v>76125</v>
-      </c>
-      <c r="H32" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I32" s="67" t="n">
-        <v>75</v>
-      </c>
-      <c r="J32" s="67" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K32" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L32" s="69" t="inlineStr">
-        <is>
-          <t>A construction worker has died at the site of the Denver Broncos' new training facility. The facility is nearing completion with a budget of $175 million.</t>
-        </is>
-      </c>
-      <c r="M32" s="69" t="inlineStr">
-        <is>
-          <t>This project represents a significant investment in the Broncos' infrastructure, which may lead to future opportunities for aluminum railings and structural components. The completion of the facility could increase demand for safety and aesthetic enhancements.</t>
-        </is>
-      </c>
-      <c r="N32" s="69" t="inlineStr">
-        <is>
-          <t>The article confirms that the Denver Broncos are finishing work on their new training facility.</t>
-        </is>
-      </c>
-      <c r="O32" s="69" t="inlineStr"/>
-      <c r="P32" s="68" t="inlineStr">
-        <is>
-          <t>https://nypost.com/2026/06/18/sports/construction-worker-dies-at-site-of-broncos-175m-training-facility/</t>
-        </is>
-      </c>
-      <c r="Q32" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R32" s="67" t="inlineStr"/>
-      <c r="S32" s="67" t="inlineStr"/>
-    </row>
-    <row r="33" ht="75" customHeight="1">
-      <c r="A33" s="64" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="63" t="inlineStr">
-        <is>
-          <t>Highmark Stadium</t>
-        </is>
-      </c>
-      <c r="C33" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D33" s="63" t="inlineStr">
-        <is>
-          <t>Buffalo Bills</t>
-        </is>
-      </c>
-      <c r="E33" s="63" t="inlineStr">
-        <is>
-          <t>Orchard Park</t>
-        </is>
-      </c>
-      <c r="F33" s="64" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="G33" s="64" t="n">
-        <v>63000</v>
-      </c>
-      <c r="H33" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I33" s="64" t="n">
-        <v>20</v>
-      </c>
-      <c r="J33" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K33" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L33" s="71" t="inlineStr">
-        <is>
-          <t>The construction of the Buffalo Bills' new stadium is progressing, currently at 75% completion. This indicates that the project is in the design phase and nearing completion.</t>
-        </is>
-      </c>
-      <c r="M33" s="71" t="inlineStr">
-        <is>
-          <t>This project is significant for our aluminum railings and platforms business as it represents a large-scale construction opportunity. Engaging with the project can lead to potential contracts for our products.</t>
-        </is>
-      </c>
-      <c r="N33" s="71" t="inlineStr">
-        <is>
-          <t>The new Highmark Stadium is set to open for the 2026 season.</t>
-        </is>
-      </c>
-      <c r="O33" s="71" t="inlineStr"/>
-      <c r="P33" s="63" t="inlineStr">
-        <is>
-          <t>https://www.espn.com/nfl/story/_/id/48291577/buffalo-bills-new-highmark-stadium-bison-statues-family-circle</t>
-        </is>
-      </c>
-      <c r="Q33" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R33" s="64" t="inlineStr"/>
-      <c r="S33" s="64" t="inlineStr"/>
-    </row>
-    <row r="34" ht="75" customHeight="1">
-      <c r="A34" s="67" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="68" t="inlineStr">
-        <is>
-          <t>Beaver Stadium</t>
-        </is>
-      </c>
-      <c r="C34" s="67" t="inlineStr">
-        <is>
-          <t>NCAA</t>
-        </is>
-      </c>
-      <c r="D34" s="68" t="inlineStr">
-        <is>
-          <t>Penn State</t>
-        </is>
-      </c>
-      <c r="E34" s="68" t="inlineStr">
-        <is>
-          <t>College Township[f]</t>
-        </is>
-      </c>
-      <c r="F34" s="67" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="G34" s="67" t="n">
-        <v>106572</v>
-      </c>
-      <c r="H34" s="73" t="inlineStr">
-        <is>
-          <t>Tier 4 — Procurement</t>
-        </is>
-      </c>
-      <c r="I34" s="67" t="n">
-        <v>18</v>
-      </c>
-      <c r="J34" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K34" s="67" t="inlineStr">
-        <is>
-          <t>Major Renovation</t>
-        </is>
-      </c>
-      <c r="L34" s="69" t="inlineStr">
-        <is>
-          <t>Populous and Penn State Athletics have revealed new details and renderings for the revitalization of Beaver Stadium. This project aims to enhance the venue's facilities and overall experience.</t>
-        </is>
-      </c>
-      <c r="M34" s="69" t="inlineStr">
-        <is>
-          <t>This renovation could significantly improve the stadium's infrastructure, leading to increased attendance and revenue. Upgraded railings and platforms will be essential for safety and accessibility.</t>
-        </is>
-      </c>
-      <c r="N34" s="69" t="inlineStr">
-        <is>
-          <t>Construction on Beaver Stadium has reached a structural milestone with the completion of the West Tower beam.</t>
-        </is>
-      </c>
-      <c r="O34" s="69" t="inlineStr"/>
-      <c r="P34" s="68" t="inlineStr">
-        <is>
-          <t>https://www.si.com/college/pennstate/football/penn-states-beaver-stadium-renovation-reaches-lofty-milestone</t>
-        </is>
-      </c>
-      <c r="Q34" s="73" t="inlineStr">
-        <is>
-          <t>too_late</t>
-        </is>
-      </c>
-      <c r="R34" s="67" t="inlineStr"/>
-      <c r="S34" s="67" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
@@ -18725,7 +16447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18750,338 +16472,101 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="75" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B1" s="75" t="inlineStr">
+      <c r="B1" s="74" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="C1" s="75" t="inlineStr">
+      <c r="C1" s="74" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="D1" s="75" t="inlineStr">
+      <c r="D1" s="74" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="E1" s="75" t="inlineStr">
+      <c r="E1" s="74" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="F1" s="75" t="inlineStr">
+      <c r="F1" s="74" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="G1" s="75" t="inlineStr">
+      <c r="G1" s="74" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="H1" s="75" t="inlineStr">
+      <c r="H1" s="74" t="inlineStr">
         <is>
           <t>Signal Tier</t>
         </is>
       </c>
-      <c r="I1" s="75" t="inlineStr">
+      <c r="I1" s="74" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="J1" s="75" t="inlineStr">
+      <c r="J1" s="74" t="inlineStr">
         <is>
           <t>Likelihood %</t>
         </is>
       </c>
-      <c r="K1" s="75" t="inlineStr">
+      <c r="K1" s="74" t="inlineStr">
         <is>
           <t>Project Type</t>
         </is>
       </c>
-      <c r="L1" s="75" t="inlineStr">
+      <c r="L1" s="74" t="inlineStr">
         <is>
           <t>What's Happening</t>
         </is>
       </c>
-      <c r="M1" s="75" t="inlineStr">
+      <c r="M1" s="74" t="inlineStr">
         <is>
           <t>Why Priority</t>
         </is>
       </c>
-      <c r="N1" s="75" t="inlineStr">
+      <c r="N1" s="74" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="O1" s="75" t="inlineStr">
+      <c r="O1" s="74" t="inlineStr">
         <is>
           <t>Stakeholders</t>
         </is>
       </c>
-      <c r="P1" s="75" t="inlineStr">
+      <c r="P1" s="74" t="inlineStr">
         <is>
           <t>Source (Link)</t>
         </is>
       </c>
-      <c r="Q1" s="75" t="inlineStr">
+      <c r="Q1" s="74" t="inlineStr">
         <is>
           <t>Engagement</t>
         </is>
       </c>
-      <c r="R1" s="75" t="inlineStr">
+      <c r="R1" s="74" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="S1" s="75" t="inlineStr">
+      <c r="S1" s="74" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="75" customHeight="1">
-      <c r="A2" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="68" t="inlineStr">
-        <is>
-          <t>New Dallas Arena</t>
-        </is>
-      </c>
-      <c r="C2" s="67" t="inlineStr">
-        <is>
-          <t>NBA</t>
-        </is>
-      </c>
-      <c r="D2" s="68" t="inlineStr">
-        <is>
-          <t>Dallas Mavericks</t>
-        </is>
-      </c>
-      <c r="E2" s="68" t="inlineStr">
-        <is>
-          <t>Dallas</t>
-        </is>
-      </c>
-      <c r="F2" s="67" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="G2" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="65" t="inlineStr">
-        <is>
-          <t>Tier 1 — Early Rumor</t>
-        </is>
-      </c>
-      <c r="I2" s="67" t="n">
-        <v>60</v>
-      </c>
-      <c r="J2" s="67" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="K2" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L2" s="69" t="inlineStr">
-        <is>
-          <t>The Dallas Mavericks are preparing for the 2026 NBA Draft. The new arena is planned for 2031, indicating future development.</t>
-        </is>
-      </c>
-      <c r="M2" s="69" t="inlineStr">
-        <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a new sports venue. Engaging early can position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N2" s="69" t="inlineStr">
-        <is>
-          <t>The venue is confirmed as planned for 2031.</t>
-        </is>
-      </c>
-      <c r="O2" s="69" t="inlineStr"/>
-      <c r="P2" s="68" t="inlineStr">
-        <is>
-          <t>https://www.si.com/nba/mavericks/onsi/monday-dallas-mavericks-mock-final-predictions-one-day-ahead-2026-nba-draft-</t>
-        </is>
-      </c>
-      <c r="Q2" s="65" t="inlineStr">
-        <is>
-          <t>engage_now</t>
-        </is>
-      </c>
-      <c r="R2" s="67" t="inlineStr"/>
-      <c r="S2" s="67" t="inlineStr"/>
-    </row>
-    <row r="3" ht="75" customHeight="1">
-      <c r="A3" s="64" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="63" t="inlineStr">
-        <is>
-          <t>New Chiefs Stadium</t>
-        </is>
-      </c>
-      <c r="C3" s="64" t="inlineStr">
-        <is>
-          <t>NFL</t>
-        </is>
-      </c>
-      <c r="D3" s="63" t="inlineStr">
-        <is>
-          <t>Kansas City Chiefs</t>
-        </is>
-      </c>
-      <c r="E3" s="63" t="inlineStr">
-        <is>
-          <t>Kansas City</t>
-        </is>
-      </c>
-      <c r="F3" s="64" t="inlineStr">
-        <is>
-          <t>KS</t>
-        </is>
-      </c>
-      <c r="G3" s="64" t="n">
-        <v>65000</v>
-      </c>
-      <c r="H3" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I3" s="64" t="n">
-        <v>60</v>
-      </c>
-      <c r="J3" s="64" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="K3" s="64" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L3" s="71" t="inlineStr">
-        <is>
-          <t>The New Chiefs Stadium is planned for construction in 2031. This project is confirmed as part of the Kansas City Chiefs' future developments.</t>
-        </is>
-      </c>
-      <c r="M3" s="71" t="inlineStr">
-        <is>
-          <t>This project represents a significant opportunity for aluminum railings and platforms in a large venue. Engaging early can position us favorably for future contracts.</t>
-        </is>
-      </c>
-      <c r="N3" s="71" t="inlineStr">
-        <is>
-          <t>Funding for the Chiefs stadium deal was approved in December 2025.</t>
-        </is>
-      </c>
-      <c r="O3" s="71" t="inlineStr"/>
-      <c r="P3" s="63" t="inlineStr">
-        <is>
-          <t>https://www.axios.com/local/kansas-city/2026/01/21/stadiums-are-becoming-micro-cities</t>
-        </is>
-      </c>
-      <c r="Q3" s="65" t="inlineStr">
-        <is>
-          <t>engage_now</t>
-        </is>
-      </c>
-      <c r="R3" s="64" t="inlineStr"/>
-      <c r="S3" s="64" t="inlineStr"/>
-    </row>
-    <row r="4" ht="75" customHeight="1">
-      <c r="A4" s="67" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="68" t="inlineStr">
-        <is>
-          <t>New Rays Stadium†</t>
-        </is>
-      </c>
-      <c r="C4" s="67" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="D4" s="68" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="E4" s="68" t="inlineStr">
-        <is>
-          <t>Tampa</t>
-        </is>
-      </c>
-      <c r="F4" s="67" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="G4" s="67" t="n">
-        <v>31000</v>
-      </c>
-      <c r="H4" s="72" t="inlineStr">
-        <is>
-          <t>Tier 2 — Funding Committed</t>
-        </is>
-      </c>
-      <c r="I4" s="67" t="n">
-        <v>49</v>
-      </c>
-      <c r="J4" s="67" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
-      <c r="K4" s="67" t="inlineStr">
-        <is>
-          <t>New Construction</t>
-        </is>
-      </c>
-      <c r="L4" s="69" t="inlineStr">
-        <is>
-          <t>The Tampa Bay Rays are planning a new stadium set to open in 2029. This project is still in the early stages of development.</t>
-        </is>
-      </c>
-      <c r="M4" s="69" t="inlineStr">
-        <is>
-          <t>This new stadium presents a significant opportunity for aluminum railings and structural components. Engaging early can position us favorably in the bidding process.</t>
-        </is>
-      </c>
-      <c r="N4" s="69" t="inlineStr">
-        <is>
-          <t>Funding for the $2.3 billion stadium has been tentatively approved by local officials.</t>
-        </is>
-      </c>
-      <c r="O4" s="69" t="inlineStr"/>
-      <c r="P4" s="68" t="inlineStr">
-        <is>
-          <t>https://bleacherreport.com/articles/25427989-rays-new-23b-stadium-tentatively-approved-local-officials-latest-timeline-revealed</t>
-        </is>
-      </c>
-      <c r="Q4" s="65" t="inlineStr">
-        <is>
-          <t>engage_now</t>
-        </is>
-      </c>
-      <c r="R4" s="67" t="inlineStr"/>
-      <c r="S4" s="67" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
@@ -19118,62 +16603,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="76" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="B1" s="76" t="inlineStr">
+      <c r="B1" s="75" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="C1" s="76" t="inlineStr">
+      <c r="C1" s="75" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="D1" s="76" t="inlineStr">
+      <c r="D1" s="75" t="inlineStr">
         <is>
           <t>Signal Tier</t>
         </is>
       </c>
-      <c r="E1" s="76" t="inlineStr">
+      <c r="E1" s="75" t="inlineStr">
         <is>
           <t>Engagement</t>
         </is>
       </c>
-      <c r="F1" s="76" t="inlineStr">
+      <c r="F1" s="75" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="G1" s="76" t="inlineStr">
+      <c r="G1" s="75" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="H1" s="76" t="inlineStr">
+      <c r="H1" s="75" t="inlineStr">
         <is>
           <t>Organization</t>
         </is>
       </c>
-      <c r="I1" s="76" t="inlineStr">
+      <c r="I1" s="75" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="J1" s="76" t="inlineStr">
+      <c r="J1" s="75" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="K1" s="76" t="inlineStr">
+      <c r="K1" s="75" t="inlineStr">
         <is>
           <t>Contact Email</t>
         </is>
       </c>
-      <c r="L1" s="76" t="inlineStr">
+      <c r="L1" s="75" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>